<commit_message>
add a common data provider
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/testdata.xlsx
+++ b/src/test/resources/excel/testdata.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ntanga101\Documents\DataDrivenFramework\src\test\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12C7241-108B-47BE-898A-39C698166507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99C307B-925A-487A-9080-14EFA0B3F26E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8964" xr2:uid="{44533C13-292C-4F00-9C65-E2FCC555769E}"/>
   </bookViews>
   <sheets>
     <sheet name="AddCustomerTest" sheetId="1" r:id="rId1"/>
+    <sheet name="OpenAccountTest" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>firstname</t>
   </si>
@@ -60,6 +61,18 @@
   </si>
   <si>
     <t>alerttext</t>
+  </si>
+  <si>
+    <t>customer</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>Ntanganedzeni Phidzaglima</t>
+  </si>
+  <si>
+    <t>Dollar</t>
   </si>
 </sst>
 </file>
@@ -470,4 +483,33 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2C42A7E-22A1-4887-A0BD-89B3FD508A18}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>